<commit_message>
added 2026 round 5 results
</commit_message>
<xml_diff>
--- a/bonus/bonus_points.xlsx
+++ b/bonus/bonus_points.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matevass/Documents/Programming/R/darts-statistics/bonus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB82D97-53C4-1846-890B-BA0656099336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A14B06B-DA69-F949-B4C3-1ABC68FB231B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="53">
   <si>
     <t>Season</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>130</t>
+  </si>
+  <si>
+    <t>119</t>
   </si>
 </sst>
 </file>
@@ -1676,10 +1679,18 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
+      <c r="A35" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>52</v>
+      </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>

</xml_diff>